<commit_message>
build_one_file_rosetta: add N indels column and sort_by_count argument
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CXqMg6LHHkTRCFtEjwRvwQ
</commit_message>
<xml_diff>
--- a/development/one_file_rosetta_output/SP107439_rosetta.xlsx
+++ b/development/one_file_rosetta_output/SP107439_rosetta.xlsx
@@ -398,14 +398,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:E183"/>
+  <dimension ref="A1:F183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" bestFit="1" customWidth="1" hidden="false" width="17.711"/>
     <col min="2" max="2" bestFit="1" customWidth="1" hidden="false" width="18.711"/>
     <col min="3" max="3" bestFit="1" customWidth="1" hidden="false" width="16.711"/>
-    <col min="4" max="4" bestFit="1" customWidth="1" hidden="false" width="4.711"/>
-    <col min="5" max="5" bestFit="1" customWidth="1" hidden="false" width="70.711"/>
+    <col min="4" max="4" bestFit="1" customWidth="1" hidden="false" width="7.711"/>
+    <col min="5" max="5" bestFit="1" customWidth="1" hidden="false" width="4.711"/>
+    <col min="6" max="6" bestFit="1" customWidth="1" hidden="false" width="70.711"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -426,10 +427,15 @@
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
+          <t>N indels</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
           <t>Example n</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Indel in context</t>
         </is>
@@ -452,9 +458,12 @@
         </is>
       </c>
       <c r="D2" s="4">
-        <v>1</v>
-      </c>
-      <c r="E2" s="6" t="inlineStr">
+        <v>13</v>
+      </c>
+      <c r="E2" s="4">
+        <v>1</v>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -508,9 +517,12 @@
         </is>
       </c>
       <c r="D3" s="4">
+        <v>13</v>
+      </c>
+      <c r="E3" s="4">
         <v>2</v>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -564,9 +576,12 @@
         </is>
       </c>
       <c r="D4" s="4">
+        <v>13</v>
+      </c>
+      <c r="E4" s="4">
         <v>3</v>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -620,9 +635,12 @@
         </is>
       </c>
       <c r="D5" s="4">
+        <v>13</v>
+      </c>
+      <c r="E5" s="4">
         <v>4</v>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -676,9 +694,12 @@
         </is>
       </c>
       <c r="D6" s="4">
+        <v>13</v>
+      </c>
+      <c r="E6" s="4">
         <v>5</v>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -732,9 +753,12 @@
         </is>
       </c>
       <c r="D7" s="4">
-        <v>1</v>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
+        <v>10</v>
+      </c>
+      <c r="E7" s="4">
+        <v>1</v>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -788,9 +812,12 @@
         </is>
       </c>
       <c r="D8" s="4">
+        <v>10</v>
+      </c>
+      <c r="E8" s="4">
         <v>2</v>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -844,9 +871,12 @@
         </is>
       </c>
       <c r="D9" s="4">
+        <v>10</v>
+      </c>
+      <c r="E9" s="4">
         <v>3</v>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -900,9 +930,12 @@
         </is>
       </c>
       <c r="D10" s="4">
+        <v>10</v>
+      </c>
+      <c r="E10" s="4">
         <v>4</v>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -956,9 +989,12 @@
         </is>
       </c>
       <c r="D11" s="4">
-        <v>1</v>
-      </c>
-      <c r="E11" s="6" t="inlineStr">
+        <v>2</v>
+      </c>
+      <c r="E11" s="4">
+        <v>1</v>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <r>
             <rPr/>
@@ -984,9 +1020,12 @@
         </is>
       </c>
       <c r="D12" s="4">
-        <v>1</v>
-      </c>
-      <c r="E12" s="6" t="inlineStr">
+        <v>5</v>
+      </c>
+      <c r="E12" s="4">
+        <v>1</v>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1040,9 +1079,12 @@
         </is>
       </c>
       <c r="D13" s="4">
+        <v>5</v>
+      </c>
+      <c r="E13" s="4">
         <v>2</v>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1096,9 +1138,12 @@
         </is>
       </c>
       <c r="D14" s="4">
+        <v>5</v>
+      </c>
+      <c r="E14" s="4">
         <v>3</v>
       </c>
-      <c r="E14" s="6" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1152,9 +1197,12 @@
         </is>
       </c>
       <c r="D15" s="4">
+        <v>5</v>
+      </c>
+      <c r="E15" s="4">
         <v>4</v>
       </c>
-      <c r="E15" s="6" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1208,9 +1256,12 @@
         </is>
       </c>
       <c r="D16" s="4">
-        <v>1</v>
-      </c>
-      <c r="E16" s="6" t="inlineStr">
+        <v>7</v>
+      </c>
+      <c r="E16" s="4">
+        <v>1</v>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1264,9 +1315,12 @@
         </is>
       </c>
       <c r="D17" s="4">
+        <v>7</v>
+      </c>
+      <c r="E17" s="4">
         <v>2</v>
       </c>
-      <c r="E17" s="6" t="inlineStr">
+      <c r="F17" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1320,9 +1374,12 @@
         </is>
       </c>
       <c r="D18" s="4">
+        <v>7</v>
+      </c>
+      <c r="E18" s="4">
         <v>3</v>
       </c>
-      <c r="E18" s="6" t="inlineStr">
+      <c r="F18" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1376,9 +1433,12 @@
         </is>
       </c>
       <c r="D19" s="4">
-        <v>1</v>
-      </c>
-      <c r="E19" s="6" t="inlineStr">
+        <v>7</v>
+      </c>
+      <c r="E19" s="4">
+        <v>1</v>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1432,9 +1492,12 @@
         </is>
       </c>
       <c r="D20" s="4">
+        <v>7</v>
+      </c>
+      <c r="E20" s="4">
         <v>2</v>
       </c>
-      <c r="E20" s="6" t="inlineStr">
+      <c r="F20" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1488,9 +1551,12 @@
         </is>
       </c>
       <c r="D21" s="4">
+        <v>7</v>
+      </c>
+      <c r="E21" s="4">
         <v>3</v>
       </c>
-      <c r="E21" s="6" t="inlineStr">
+      <c r="F21" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1546,7 +1612,10 @@
       <c r="D22" s="4">
         <v>1</v>
       </c>
-      <c r="E22" s="6" t="inlineStr">
+      <c r="E22" s="4">
+        <v>1</v>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1615,9 +1684,12 @@
         </is>
       </c>
       <c r="D23" s="4">
-        <v>1</v>
-      </c>
-      <c r="E23" s="6" t="inlineStr">
+        <v>13</v>
+      </c>
+      <c r="E23" s="4">
+        <v>1</v>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1671,9 +1743,12 @@
         </is>
       </c>
       <c r="D24" s="4">
+        <v>13</v>
+      </c>
+      <c r="E24" s="4">
         <v>2</v>
       </c>
-      <c r="E24" s="6" t="inlineStr">
+      <c r="F24" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1727,9 +1802,12 @@
         </is>
       </c>
       <c r="D25" s="4">
+        <v>13</v>
+      </c>
+      <c r="E25" s="4">
         <v>3</v>
       </c>
-      <c r="E25" s="6" t="inlineStr">
+      <c r="F25" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1783,9 +1861,12 @@
         </is>
       </c>
       <c r="D26" s="4">
+        <v>13</v>
+      </c>
+      <c r="E26" s="4">
         <v>4</v>
       </c>
-      <c r="E26" s="6" t="inlineStr">
+      <c r="F26" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1839,9 +1920,12 @@
         </is>
       </c>
       <c r="D27" s="4">
+        <v>13</v>
+      </c>
+      <c r="E27" s="4">
         <v>5</v>
       </c>
-      <c r="E27" s="6" t="inlineStr">
+      <c r="F27" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1895,9 +1979,12 @@
         </is>
       </c>
       <c r="D28" s="4">
-        <v>1</v>
-      </c>
-      <c r="E28" s="6" t="inlineStr">
+        <v>4</v>
+      </c>
+      <c r="E28" s="4">
+        <v>1</v>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1951,9 +2038,12 @@
         </is>
       </c>
       <c r="D29" s="4">
-        <v>1</v>
-      </c>
-      <c r="E29" s="6" t="inlineStr">
+        <v>9</v>
+      </c>
+      <c r="E29" s="4">
+        <v>1</v>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2007,9 +2097,12 @@
         </is>
       </c>
       <c r="D30" s="4">
+        <v>9</v>
+      </c>
+      <c r="E30" s="4">
         <v>2</v>
       </c>
-      <c r="E30" s="6" t="inlineStr">
+      <c r="F30" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2063,9 +2156,12 @@
         </is>
       </c>
       <c r="D31" s="4">
+        <v>9</v>
+      </c>
+      <c r="E31" s="4">
         <v>3</v>
       </c>
-      <c r="E31" s="6" t="inlineStr">
+      <c r="F31" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2119,9 +2215,12 @@
         </is>
       </c>
       <c r="D32" s="4">
+        <v>9</v>
+      </c>
+      <c r="E32" s="4">
         <v>4</v>
       </c>
-      <c r="E32" s="6" t="inlineStr">
+      <c r="F32" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2175,9 +2274,12 @@
         </is>
       </c>
       <c r="D33" s="4">
+        <v>9</v>
+      </c>
+      <c r="E33" s="4">
         <v>5</v>
       </c>
-      <c r="E33" s="6" t="inlineStr">
+      <c r="F33" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2231,9 +2333,12 @@
         </is>
       </c>
       <c r="D34" s="4">
-        <v>1</v>
-      </c>
-      <c r="E34" s="6" t="inlineStr">
+        <v>4</v>
+      </c>
+      <c r="E34" s="4">
+        <v>1</v>
+      </c>
+      <c r="F34" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2294,9 +2399,12 @@
         </is>
       </c>
       <c r="D35" s="4">
+        <v>4</v>
+      </c>
+      <c r="E35" s="4">
         <v>2</v>
       </c>
-      <c r="E35" s="6" t="inlineStr">
+      <c r="F35" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2359,7 +2467,10 @@
       <c r="D36" s="4">
         <v>1</v>
       </c>
-      <c r="E36" s="6" t="inlineStr">
+      <c r="E36" s="4">
+        <v>1</v>
+      </c>
+      <c r="F36" s="6" t="inlineStr">
         <is>
           <r>
             <rPr/>
@@ -2387,7 +2498,10 @@
       <c r="D37" s="4">
         <v>1</v>
       </c>
-      <c r="E37" s="6" t="inlineStr">
+      <c r="E37" s="4">
+        <v>1</v>
+      </c>
+      <c r="F37" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2473,7 +2587,10 @@
       <c r="D38" s="4">
         <v>1</v>
       </c>
-      <c r="E38" s="6" t="inlineStr">
+      <c r="E38" s="4">
+        <v>1</v>
+      </c>
+      <c r="F38" s="6" t="inlineStr">
         <is>
           <r>
             <rPr/>
@@ -2501,7 +2618,10 @@
       <c r="D39" s="4">
         <v>1</v>
       </c>
-      <c r="E39" s="6" t="inlineStr">
+      <c r="E39" s="4">
+        <v>1</v>
+      </c>
+      <c r="F39" s="6" t="inlineStr">
         <is>
           <r>
             <rPr/>
@@ -2527,9 +2647,12 @@
         </is>
       </c>
       <c r="D40" s="4">
-        <v>1</v>
-      </c>
-      <c r="E40" s="6" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="E40" s="4">
+        <v>1</v>
+      </c>
+      <c r="F40" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2628,9 +2751,12 @@
         </is>
       </c>
       <c r="D41" s="4">
+        <v>3</v>
+      </c>
+      <c r="E41" s="4">
         <v>2</v>
       </c>
-      <c r="E41" s="6" t="inlineStr">
+      <c r="F41" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2731,7 +2857,10 @@
       <c r="D42" s="4">
         <v>1</v>
       </c>
-      <c r="E42" s="6" t="inlineStr">
+      <c r="E42" s="4">
+        <v>1</v>
+      </c>
+      <c r="F42" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2839,7 +2968,10 @@
       <c r="D43" s="4">
         <v>1</v>
       </c>
-      <c r="E43" s="6" t="inlineStr">
+      <c r="E43" s="4">
+        <v>1</v>
+      </c>
+      <c r="F43" s="6" t="inlineStr">
         <is>
           <r>
             <rPr/>
@@ -2865,9 +2997,12 @@
         </is>
       </c>
       <c r="D44" s="4">
-        <v>1</v>
-      </c>
-      <c r="E44" s="6" t="inlineStr">
+        <v>5</v>
+      </c>
+      <c r="E44" s="4">
+        <v>1</v>
+      </c>
+      <c r="F44" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2921,9 +3056,12 @@
         </is>
       </c>
       <c r="D45" s="4">
+        <v>5</v>
+      </c>
+      <c r="E45" s="4">
         <v>2</v>
       </c>
-      <c r="E45" s="6" t="inlineStr">
+      <c r="F45" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2977,9 +3115,12 @@
         </is>
       </c>
       <c r="D46" s="4">
+        <v>5</v>
+      </c>
+      <c r="E46" s="4">
         <v>3</v>
       </c>
-      <c r="E46" s="6" t="inlineStr">
+      <c r="F46" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3035,7 +3176,10 @@
       <c r="D47" s="4">
         <v>1</v>
       </c>
-      <c r="E47" s="6" t="inlineStr">
+      <c r="E47" s="4">
+        <v>1</v>
+      </c>
+      <c r="F47" s="6" t="inlineStr">
         <is>
           <r>
             <rPr/>
@@ -3063,7 +3207,10 @@
       <c r="D48" s="4">
         <v>1</v>
       </c>
-      <c r="E48" s="6" t="inlineStr">
+      <c r="E48" s="4">
+        <v>1</v>
+      </c>
+      <c r="F48" s="6" t="inlineStr">
         <is>
           <r>
             <rPr/>
@@ -3091,7 +3238,10 @@
       <c r="D49" s="4">
         <v>1</v>
       </c>
-      <c r="E49" s="6" t="inlineStr">
+      <c r="E49" s="4">
+        <v>1</v>
+      </c>
+      <c r="F49" s="6" t="inlineStr">
         <is>
           <r>
             <rPr/>
@@ -3119,7 +3269,10 @@
       <c r="D50" s="4">
         <v>1</v>
       </c>
-      <c r="E50" s="6" t="inlineStr">
+      <c r="E50" s="4">
+        <v>1</v>
+      </c>
+      <c r="F50" s="6" t="inlineStr">
         <is>
           <r>
             <rPr/>
@@ -3145,9 +3298,12 @@
         </is>
       </c>
       <c r="D51" s="4">
-        <v>1</v>
-      </c>
-      <c r="E51" s="6" t="inlineStr">
+        <v>2</v>
+      </c>
+      <c r="E51" s="4">
+        <v>1</v>
+      </c>
+      <c r="F51" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3218,7 +3374,10 @@
       <c r="D52" s="4">
         <v>2</v>
       </c>
-      <c r="E52" s="6" t="inlineStr">
+      <c r="E52" s="4">
+        <v>2</v>
+      </c>
+      <c r="F52" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3289,7 +3448,10 @@
       <c r="D53" s="4">
         <v>1</v>
       </c>
-      <c r="E53" s="6" t="inlineStr">
+      <c r="E53" s="4">
+        <v>1</v>
+      </c>
+      <c r="F53" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3367,7 +3529,10 @@
       <c r="D54" s="4">
         <v>1</v>
       </c>
-      <c r="E54" s="6" t="inlineStr">
+      <c r="E54" s="4">
+        <v>1</v>
+      </c>
+      <c r="F54" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3445,7 +3610,10 @@
       <c r="D55" s="4">
         <v>1</v>
       </c>
-      <c r="E55" s="6" t="inlineStr">
+      <c r="E55" s="4">
+        <v>1</v>
+      </c>
+      <c r="F55" s="6" t="inlineStr">
         <is>
           <r>
             <rPr/>
@@ -3473,7 +3641,10 @@
       <c r="D56" s="4">
         <v>1</v>
       </c>
-      <c r="E56" s="6" t="inlineStr">
+      <c r="E56" s="4">
+        <v>1</v>
+      </c>
+      <c r="F56" s="6" t="inlineStr">
         <is>
           <r>
             <rPr/>
@@ -3499,9 +3670,12 @@
         </is>
       </c>
       <c r="D57" s="4">
-        <v>1</v>
-      </c>
-      <c r="E57" s="6" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="E57" s="4">
+        <v>1</v>
+      </c>
+      <c r="F57" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3555,9 +3729,12 @@
         </is>
       </c>
       <c r="D58" s="4">
+        <v>3</v>
+      </c>
+      <c r="E58" s="4">
         <v>2</v>
       </c>
-      <c r="E58" s="6" t="inlineStr">
+      <c r="F58" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3613,7 +3790,10 @@
       <c r="D59" s="4">
         <v>3</v>
       </c>
-      <c r="E59" s="6" t="inlineStr">
+      <c r="E59" s="4">
+        <v>3</v>
+      </c>
+      <c r="F59" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3667,9 +3847,12 @@
         </is>
       </c>
       <c r="D60" s="4">
-        <v>1</v>
-      </c>
-      <c r="E60" s="6" t="inlineStr">
+        <v>2</v>
+      </c>
+      <c r="E60" s="4">
+        <v>1</v>
+      </c>
+      <c r="F60" s="6" t="inlineStr">
         <is>
           <r>
             <rPr/>
@@ -3697,7 +3880,10 @@
       <c r="D61" s="4">
         <v>1</v>
       </c>
-      <c r="E61" s="6" t="inlineStr">
+      <c r="E61" s="4">
+        <v>1</v>
+      </c>
+      <c r="F61" s="6" t="inlineStr">
         <is>
           <r>
             <rPr/>
@@ -3725,7 +3911,10 @@
       <c r="D62" s="4">
         <v>1</v>
       </c>
-      <c r="E62" s="6" t="inlineStr">
+      <c r="E62" s="4">
+        <v>1</v>
+      </c>
+      <c r="F62" s="6" t="inlineStr">
         <is>
           <r>
             <rPr/>
@@ -3753,7 +3942,10 @@
       <c r="D63" s="4">
         <v>1</v>
       </c>
-      <c r="E63" s="6" t="inlineStr">
+      <c r="E63" s="4">
+        <v>1</v>
+      </c>
+      <c r="F63" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3831,7 +4023,10 @@
       <c r="D64" s="4">
         <v>1</v>
       </c>
-      <c r="E64" s="6" t="inlineStr">
+      <c r="E64" s="4">
+        <v>1</v>
+      </c>
+      <c r="F64" s="6" t="inlineStr">
         <is>
           <r>
             <rPr/>
@@ -3857,9 +4052,12 @@
         </is>
       </c>
       <c r="D65" s="4">
-        <v>1</v>
-      </c>
-      <c r="E65" s="6" t="inlineStr">
+        <v>11</v>
+      </c>
+      <c r="E65" s="4">
+        <v>1</v>
+      </c>
+      <c r="F65" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3913,9 +4111,12 @@
         </is>
       </c>
       <c r="D66" s="4">
+        <v>11</v>
+      </c>
+      <c r="E66" s="4">
         <v>2</v>
       </c>
-      <c r="E66" s="6" t="inlineStr">
+      <c r="F66" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3969,9 +4170,12 @@
         </is>
       </c>
       <c r="D67" s="4">
+        <v>11</v>
+      </c>
+      <c r="E67" s="4">
         <v>3</v>
       </c>
-      <c r="E67" s="6" t="inlineStr">
+      <c r="F67" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4025,9 +4229,12 @@
         </is>
       </c>
       <c r="D68" s="4">
+        <v>11</v>
+      </c>
+      <c r="E68" s="4">
         <v>4</v>
       </c>
-      <c r="E68" s="6" t="inlineStr">
+      <c r="F68" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4081,9 +4288,12 @@
         </is>
       </c>
       <c r="D69" s="4">
+        <v>11</v>
+      </c>
+      <c r="E69" s="4">
         <v>5</v>
       </c>
-      <c r="E69" s="6" t="inlineStr">
+      <c r="F69" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4139,7 +4349,10 @@
       <c r="D70" s="4">
         <v>1</v>
       </c>
-      <c r="E70" s="6" t="inlineStr">
+      <c r="E70" s="4">
+        <v>1</v>
+      </c>
+      <c r="F70" s="6" t="inlineStr">
         <is>
           <r>
             <rPr/>
@@ -4165,9 +4378,12 @@
         </is>
       </c>
       <c r="D71" s="4">
-        <v>1</v>
-      </c>
-      <c r="E71" s="6" t="inlineStr">
+        <v>8</v>
+      </c>
+      <c r="E71" s="4">
+        <v>1</v>
+      </c>
+      <c r="F71" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4221,9 +4437,12 @@
         </is>
       </c>
       <c r="D72" s="4">
+        <v>8</v>
+      </c>
+      <c r="E72" s="4">
         <v>2</v>
       </c>
-      <c r="E72" s="6" t="inlineStr">
+      <c r="F72" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4277,9 +4496,12 @@
         </is>
       </c>
       <c r="D73" s="4">
+        <v>8</v>
+      </c>
+      <c r="E73" s="4">
         <v>3</v>
       </c>
-      <c r="E73" s="6" t="inlineStr">
+      <c r="F73" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4333,9 +4555,12 @@
         </is>
       </c>
       <c r="D74" s="4">
+        <v>8</v>
+      </c>
+      <c r="E74" s="4">
         <v>4</v>
       </c>
-      <c r="E74" s="6" t="inlineStr">
+      <c r="F74" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4391,7 +4616,10 @@
       <c r="D75" s="4">
         <v>1</v>
       </c>
-      <c r="E75" s="6" t="inlineStr">
+      <c r="E75" s="4">
+        <v>1</v>
+      </c>
+      <c r="F75" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4452,9 +4680,12 @@
         </is>
       </c>
       <c r="D76" s="4">
-        <v>1</v>
-      </c>
-      <c r="E76" s="6" t="inlineStr">
+        <v>2</v>
+      </c>
+      <c r="E76" s="4">
+        <v>1</v>
+      </c>
+      <c r="F76" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4508,9 +4739,12 @@
         </is>
       </c>
       <c r="D77" s="4">
-        <v>1</v>
-      </c>
-      <c r="E77" s="6" t="inlineStr">
+        <v>2</v>
+      </c>
+      <c r="E77" s="4">
+        <v>1</v>
+      </c>
+      <c r="F77" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4566,7 +4800,10 @@
       <c r="D78" s="4">
         <v>2</v>
       </c>
-      <c r="E78" s="6" t="inlineStr">
+      <c r="E78" s="4">
+        <v>2</v>
+      </c>
+      <c r="F78" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4620,9 +4857,12 @@
         </is>
       </c>
       <c r="D79" s="4">
-        <v>1</v>
-      </c>
-      <c r="E79" s="6" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="E79" s="4">
+        <v>1</v>
+      </c>
+      <c r="F79" s="6" t="inlineStr">
         <is>
           <r>
             <rPr/>
@@ -4648,9 +4888,12 @@
         </is>
       </c>
       <c r="D80" s="4">
-        <v>1</v>
-      </c>
-      <c r="E80" s="6" t="inlineStr">
+        <v>10</v>
+      </c>
+      <c r="E80" s="4">
+        <v>1</v>
+      </c>
+      <c r="F80" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4704,9 +4947,12 @@
         </is>
       </c>
       <c r="D81" s="4">
+        <v>10</v>
+      </c>
+      <c r="E81" s="4">
         <v>2</v>
       </c>
-      <c r="E81" s="6" t="inlineStr">
+      <c r="F81" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4760,9 +5006,12 @@
         </is>
       </c>
       <c r="D82" s="4">
+        <v>10</v>
+      </c>
+      <c r="E82" s="4">
         <v>3</v>
       </c>
-      <c r="E82" s="6" t="inlineStr">
+      <c r="F82" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4816,9 +5065,12 @@
         </is>
       </c>
       <c r="D83" s="4">
-        <v>1</v>
-      </c>
-      <c r="E83" s="6" t="inlineStr">
+        <v>17</v>
+      </c>
+      <c r="E83" s="4">
+        <v>1</v>
+      </c>
+      <c r="F83" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4872,9 +5124,12 @@
         </is>
       </c>
       <c r="D84" s="4">
+        <v>17</v>
+      </c>
+      <c r="E84" s="4">
         <v>2</v>
       </c>
-      <c r="E84" s="6" t="inlineStr">
+      <c r="F84" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4928,9 +5183,12 @@
         </is>
       </c>
       <c r="D85" s="4">
+        <v>17</v>
+      </c>
+      <c r="E85" s="4">
         <v>3</v>
       </c>
-      <c r="E85" s="6" t="inlineStr">
+      <c r="F85" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4984,9 +5242,12 @@
         </is>
       </c>
       <c r="D86" s="4">
+        <v>17</v>
+      </c>
+      <c r="E86" s="4">
         <v>4</v>
       </c>
-      <c r="E86" s="6" t="inlineStr">
+      <c r="F86" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -5040,9 +5301,12 @@
         </is>
       </c>
       <c r="D87" s="4">
+        <v>17</v>
+      </c>
+      <c r="E87" s="4">
         <v>5</v>
       </c>
-      <c r="E87" s="6" t="inlineStr">
+      <c r="F87" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -5096,9 +5360,12 @@
         </is>
       </c>
       <c r="D88" s="4">
-        <v>1</v>
-      </c>
-      <c r="E88" s="6" t="inlineStr">
+        <v>4</v>
+      </c>
+      <c r="E88" s="4">
+        <v>1</v>
+      </c>
+      <c r="F88" s="6" t="inlineStr">
         <is>
           <r>
             <rPr/>
@@ -5124,9 +5391,12 @@
         </is>
       </c>
       <c r="D89" s="4">
-        <v>1</v>
-      </c>
-      <c r="E89" s="6" t="inlineStr">
+        <v>8</v>
+      </c>
+      <c r="E89" s="4">
+        <v>1</v>
+      </c>
+      <c r="F89" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -5180,9 +5450,12 @@
         </is>
       </c>
       <c r="D90" s="4">
+        <v>8</v>
+      </c>
+      <c r="E90" s="4">
         <v>2</v>
       </c>
-      <c r="E90" s="6" t="inlineStr">
+      <c r="F90" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -5236,9 +5509,12 @@
         </is>
       </c>
       <c r="D91" s="4">
+        <v>8</v>
+      </c>
+      <c r="E91" s="4">
         <v>3</v>
       </c>
-      <c r="E91" s="6" t="inlineStr">
+      <c r="F91" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -5292,9 +5568,12 @@
         </is>
       </c>
       <c r="D92" s="4">
+        <v>8</v>
+      </c>
+      <c r="E92" s="4">
         <v>4</v>
       </c>
-      <c r="E92" s="6" t="inlineStr">
+      <c r="F92" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -5348,9 +5627,12 @@
         </is>
       </c>
       <c r="D93" s="4">
-        <v>1</v>
-      </c>
-      <c r="E93" s="6" t="inlineStr">
+        <v>4</v>
+      </c>
+      <c r="E93" s="4">
+        <v>1</v>
+      </c>
+      <c r="F93" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -5411,9 +5693,12 @@
         </is>
       </c>
       <c r="D94" s="4">
+        <v>4</v>
+      </c>
+      <c r="E94" s="4">
         <v>2</v>
       </c>
-      <c r="E94" s="6" t="inlineStr">
+      <c r="F94" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -5476,7 +5761,10 @@
       <c r="D95" s="4">
         <v>1</v>
       </c>
-      <c r="E95" s="6" t="inlineStr">
+      <c r="E95" s="4">
+        <v>1</v>
+      </c>
+      <c r="F95" s="6" t="inlineStr">
         <is>
           <r>
             <rPr/>
@@ -5502,9 +5790,12 @@
         </is>
       </c>
       <c r="D96" s="4">
-        <v>1</v>
-      </c>
-      <c r="E96" s="6" t="inlineStr">
+        <v>2</v>
+      </c>
+      <c r="E96" s="4">
+        <v>1</v>
+      </c>
+      <c r="F96" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -5567,7 +5858,10 @@
       <c r="D97" s="4">
         <v>1</v>
       </c>
-      <c r="E97" s="6" t="inlineStr">
+      <c r="E97" s="4">
+        <v>1</v>
+      </c>
+      <c r="F97" s="6" t="inlineStr">
         <is>
           <r>
             <rPr/>
@@ -5595,7 +5889,10 @@
       <c r="D98" s="4">
         <v>1</v>
       </c>
-      <c r="E98" s="6" t="inlineStr">
+      <c r="E98" s="4">
+        <v>1</v>
+      </c>
+      <c r="F98" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -5673,7 +5970,10 @@
       <c r="D99" s="4">
         <v>1</v>
       </c>
-      <c r="E99" s="6" t="inlineStr">
+      <c r="E99" s="4">
+        <v>1</v>
+      </c>
+      <c r="F99" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -5751,7 +6051,10 @@
       <c r="D100" s="4">
         <v>1</v>
       </c>
-      <c r="E100" s="6" t="inlineStr">
+      <c r="E100" s="4">
+        <v>1</v>
+      </c>
+      <c r="F100" s="6" t="inlineStr">
         <is>
           <r>
             <rPr/>
@@ -5777,9 +6080,12 @@
         </is>
       </c>
       <c r="D101" s="4">
-        <v>1</v>
-      </c>
-      <c r="E101" s="6" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="E101" s="4">
+        <v>1</v>
+      </c>
+      <c r="F101" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -5878,9 +6184,12 @@
         </is>
       </c>
       <c r="D102" s="4">
-        <v>1</v>
-      </c>
-      <c r="E102" s="6" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="E102" s="4">
+        <v>1</v>
+      </c>
+      <c r="F102" s="6" t="inlineStr">
         <is>
           <r>
             <rPr/>
@@ -5906,9 +6215,12 @@
         </is>
       </c>
       <c r="D103" s="4">
-        <v>1</v>
-      </c>
-      <c r="E103" s="6" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="E103" s="4">
+        <v>1</v>
+      </c>
+      <c r="F103" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -6014,9 +6326,12 @@
         </is>
       </c>
       <c r="D104" s="4">
+        <v>3</v>
+      </c>
+      <c r="E104" s="4">
         <v>2</v>
       </c>
-      <c r="E104" s="6" t="inlineStr">
+      <c r="F104" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -6124,7 +6439,10 @@
       <c r="D105" s="4">
         <v>3</v>
       </c>
-      <c r="E105" s="6" t="inlineStr">
+      <c r="E105" s="4">
+        <v>3</v>
+      </c>
+      <c r="F105" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -6230,9 +6548,12 @@
         </is>
       </c>
       <c r="D106" s="4">
-        <v>1</v>
-      </c>
-      <c r="E106" s="6" t="inlineStr">
+        <v>2</v>
+      </c>
+      <c r="E106" s="4">
+        <v>1</v>
+      </c>
+      <c r="F106" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -6348,7 +6669,10 @@
       <c r="D107" s="4">
         <v>1</v>
       </c>
-      <c r="E107" s="6" t="inlineStr">
+      <c r="E107" s="4">
+        <v>1</v>
+      </c>
+      <c r="F107" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -6464,7 +6788,10 @@
       <c r="D108" s="4">
         <v>1</v>
       </c>
-      <c r="E108" s="6" t="inlineStr">
+      <c r="E108" s="4">
+        <v>1</v>
+      </c>
+      <c r="F108" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -6587,7 +6914,10 @@
       <c r="D109" s="4">
         <v>1</v>
       </c>
-      <c r="E109" s="6" t="inlineStr">
+      <c r="E109" s="4">
+        <v>1</v>
+      </c>
+      <c r="F109" s="6" t="inlineStr">
         <is>
           <r>
             <rPr/>
@@ -6613,9 +6943,12 @@
         </is>
       </c>
       <c r="D110" s="4">
-        <v>1</v>
-      </c>
-      <c r="E110" s="6" t="inlineStr">
+        <v>4</v>
+      </c>
+      <c r="E110" s="4">
+        <v>1</v>
+      </c>
+      <c r="F110" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -6669,9 +7002,12 @@
         </is>
       </c>
       <c r="D111" s="4">
+        <v>4</v>
+      </c>
+      <c r="E111" s="4">
         <v>2</v>
       </c>
-      <c r="E111" s="6" t="inlineStr">
+      <c r="F111" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -6725,9 +7061,12 @@
         </is>
       </c>
       <c r="D112" s="4">
-        <v>1</v>
-      </c>
-      <c r="E112" s="6" t="inlineStr">
+        <v>4</v>
+      </c>
+      <c r="E112" s="4">
+        <v>1</v>
+      </c>
+      <c r="F112" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -6781,9 +7120,12 @@
         </is>
       </c>
       <c r="D113" s="4">
+        <v>4</v>
+      </c>
+      <c r="E113" s="4">
         <v>2</v>
       </c>
-      <c r="E113" s="6" t="inlineStr">
+      <c r="F113" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -6839,7 +7181,10 @@
       <c r="D114" s="4">
         <v>1</v>
       </c>
-      <c r="E114" s="6" t="inlineStr">
+      <c r="E114" s="4">
+        <v>1</v>
+      </c>
+      <c r="F114" s="6" t="inlineStr">
         <is>
           <r>
             <rPr/>
@@ -6867,7 +7212,10 @@
       <c r="D115" s="4">
         <v>1</v>
       </c>
-      <c r="E115" s="6" t="inlineStr">
+      <c r="E115" s="4">
+        <v>1</v>
+      </c>
+      <c r="F115" s="6" t="inlineStr">
         <is>
           <r>
             <rPr/>
@@ -6895,7 +7243,10 @@
       <c r="D116" s="4">
         <v>1</v>
       </c>
-      <c r="E116" s="6" t="inlineStr">
+      <c r="E116" s="4">
+        <v>1</v>
+      </c>
+      <c r="F116" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -6988,7 +7339,10 @@
       <c r="D117" s="4">
         <v>1</v>
       </c>
-      <c r="E117" s="6" t="inlineStr">
+      <c r="E117" s="4">
+        <v>1</v>
+      </c>
+      <c r="F117" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -7087,9 +7441,12 @@
         </is>
       </c>
       <c r="D118" s="4">
-        <v>1</v>
-      </c>
-      <c r="E118" s="6" t="inlineStr">
+        <v>2</v>
+      </c>
+      <c r="E118" s="4">
+        <v>1</v>
+      </c>
+      <c r="F118" s="6" t="inlineStr">
         <is>
           <r>
             <rPr/>
@@ -7117,7 +7474,10 @@
       <c r="D119" s="4">
         <v>1</v>
       </c>
-      <c r="E119" s="6" t="inlineStr">
+      <c r="E119" s="4">
+        <v>1</v>
+      </c>
+      <c r="F119" s="6" t="inlineStr">
         <is>
           <r>
             <rPr/>
@@ -7145,7 +7505,10 @@
       <c r="D120" s="4">
         <v>1</v>
       </c>
-      <c r="E120" s="6" t="inlineStr">
+      <c r="E120" s="4">
+        <v>1</v>
+      </c>
+      <c r="F120" s="6" t="inlineStr">
         <is>
           <r>
             <rPr/>
@@ -7171,9 +7534,12 @@
         </is>
       </c>
       <c r="D121" s="4">
-        <v>1</v>
-      </c>
-      <c r="E121" s="6" t="inlineStr">
+        <v>2</v>
+      </c>
+      <c r="E121" s="4">
+        <v>1</v>
+      </c>
+      <c r="F121" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -7287,9 +7653,12 @@
         </is>
       </c>
       <c r="D122" s="4">
-        <v>1</v>
-      </c>
-      <c r="E122" s="6" t="inlineStr">
+        <v>2</v>
+      </c>
+      <c r="E122" s="4">
+        <v>1</v>
+      </c>
+      <c r="F122" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -7410,9 +7779,12 @@
         </is>
       </c>
       <c r="D123" s="4">
-        <v>1</v>
-      </c>
-      <c r="E123" s="6" t="inlineStr">
+        <v>8</v>
+      </c>
+      <c r="E123" s="4">
+        <v>1</v>
+      </c>
+      <c r="F123" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -7466,9 +7838,12 @@
         </is>
       </c>
       <c r="D124" s="4">
+        <v>8</v>
+      </c>
+      <c r="E124" s="4">
         <v>2</v>
       </c>
-      <c r="E124" s="6" t="inlineStr">
+      <c r="F124" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -7522,9 +7897,12 @@
         </is>
       </c>
       <c r="D125" s="4">
+        <v>8</v>
+      </c>
+      <c r="E125" s="4">
         <v>3</v>
       </c>
-      <c r="E125" s="6" t="inlineStr">
+      <c r="F125" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -7578,9 +7956,12 @@
         </is>
       </c>
       <c r="D126" s="4">
-        <v>1</v>
-      </c>
-      <c r="E126" s="6" t="inlineStr">
+        <v>7</v>
+      </c>
+      <c r="E126" s="4">
+        <v>1</v>
+      </c>
+      <c r="F126" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -7634,9 +8015,12 @@
         </is>
       </c>
       <c r="D127" s="4">
+        <v>7</v>
+      </c>
+      <c r="E127" s="4">
         <v>2</v>
       </c>
-      <c r="E127" s="6" t="inlineStr">
+      <c r="F127" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -7690,9 +8074,12 @@
         </is>
       </c>
       <c r="D128" s="4">
+        <v>7</v>
+      </c>
+      <c r="E128" s="4">
         <v>3</v>
       </c>
-      <c r="E128" s="6" t="inlineStr">
+      <c r="F128" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -7746,9 +8133,12 @@
         </is>
       </c>
       <c r="D129" s="4">
+        <v>7</v>
+      </c>
+      <c r="E129" s="4">
         <v>4</v>
       </c>
-      <c r="E129" s="6" t="inlineStr">
+      <c r="F129" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -7802,9 +8192,12 @@
         </is>
       </c>
       <c r="D130" s="4">
+        <v>7</v>
+      </c>
+      <c r="E130" s="4">
         <v>5</v>
       </c>
-      <c r="E130" s="6" t="inlineStr">
+      <c r="F130" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -7858,9 +8251,12 @@
         </is>
       </c>
       <c r="D131" s="4">
-        <v>1</v>
-      </c>
-      <c r="E131" s="6" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="E131" s="4">
+        <v>1</v>
+      </c>
+      <c r="F131" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -7914,9 +8310,12 @@
         </is>
       </c>
       <c r="D132" s="4">
+        <v>3</v>
+      </c>
+      <c r="E132" s="4">
         <v>2</v>
       </c>
-      <c r="E132" s="6" t="inlineStr">
+      <c r="F132" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -7972,7 +8371,10 @@
       <c r="D133" s="4">
         <v>1</v>
       </c>
-      <c r="E133" s="6" t="inlineStr">
+      <c r="E133" s="4">
+        <v>1</v>
+      </c>
+      <c r="F133" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -8033,9 +8435,12 @@
         </is>
       </c>
       <c r="D134" s="4">
-        <v>1</v>
-      </c>
-      <c r="E134" s="6" t="inlineStr">
+        <v>2</v>
+      </c>
+      <c r="E134" s="4">
+        <v>1</v>
+      </c>
+      <c r="F134" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -8098,7 +8503,10 @@
       <c r="D135" s="4">
         <v>2</v>
       </c>
-      <c r="E135" s="6" t="inlineStr">
+      <c r="E135" s="4">
+        <v>2</v>
+      </c>
+      <c r="F135" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -8161,7 +8569,10 @@
       <c r="D136" s="4">
         <v>1</v>
       </c>
-      <c r="E136" s="6" t="inlineStr">
+      <c r="E136" s="4">
+        <v>1</v>
+      </c>
+      <c r="F136" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -8232,7 +8643,10 @@
       <c r="D137" s="4">
         <v>1</v>
       </c>
-      <c r="E137" s="6" t="inlineStr">
+      <c r="E137" s="4">
+        <v>1</v>
+      </c>
+      <c r="F137" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -8333,7 +8747,10 @@
       <c r="D138" s="4">
         <v>1</v>
       </c>
-      <c r="E138" s="6" t="inlineStr">
+      <c r="E138" s="4">
+        <v>1</v>
+      </c>
+      <c r="F138" s="6" t="inlineStr">
         <is>
           <r>
             <rPr/>
@@ -8361,7 +8778,10 @@
       <c r="D139" s="4">
         <v>1</v>
       </c>
-      <c r="E139" s="6" t="inlineStr">
+      <c r="E139" s="4">
+        <v>1</v>
+      </c>
+      <c r="F139" s="6" t="inlineStr">
         <is>
           <r>
             <rPr/>
@@ -8389,7 +8809,10 @@
       <c r="D140" s="4">
         <v>1</v>
       </c>
-      <c r="E140" s="6" t="inlineStr">
+      <c r="E140" s="4">
+        <v>1</v>
+      </c>
+      <c r="F140" s="6" t="inlineStr">
         <is>
           <r>
             <rPr/>
@@ -8415,9 +8838,12 @@
         </is>
       </c>
       <c r="D141" s="4">
-        <v>1</v>
-      </c>
-      <c r="E141" s="6" t="inlineStr">
+        <v>2</v>
+      </c>
+      <c r="E141" s="4">
+        <v>1</v>
+      </c>
+      <c r="F141" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -8533,7 +8959,10 @@
       <c r="D142" s="4">
         <v>2</v>
       </c>
-      <c r="E142" s="6" t="inlineStr">
+      <c r="E142" s="4">
+        <v>2</v>
+      </c>
+      <c r="F142" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -8649,7 +9078,10 @@
       <c r="D143" s="4">
         <v>1</v>
       </c>
-      <c r="E143" s="6" t="inlineStr">
+      <c r="E143" s="4">
+        <v>1</v>
+      </c>
+      <c r="F143" s="6" t="inlineStr">
         <is>
           <r>
             <rPr/>
@@ -8677,7 +9109,10 @@
       <c r="D144" s="4">
         <v>1</v>
       </c>
-      <c r="E144" s="6" t="inlineStr">
+      <c r="E144" s="4">
+        <v>1</v>
+      </c>
+      <c r="F144" s="6" t="inlineStr">
         <is>
           <r>
             <rPr/>
@@ -8705,7 +9140,10 @@
       <c r="D145" s="4">
         <v>1</v>
       </c>
-      <c r="E145" s="6" t="inlineStr">
+      <c r="E145" s="4">
+        <v>1</v>
+      </c>
+      <c r="F145" s="6" t="inlineStr">
         <is>
           <r>
             <rPr/>
@@ -8733,7 +9171,10 @@
       <c r="D146" s="4">
         <v>1</v>
       </c>
-      <c r="E146" s="6" t="inlineStr">
+      <c r="E146" s="4">
+        <v>1</v>
+      </c>
+      <c r="F146" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -8787,9 +9228,12 @@
         </is>
       </c>
       <c r="D147" s="4">
-        <v>1</v>
-      </c>
-      <c r="E147" s="6" t="inlineStr">
+        <v>7</v>
+      </c>
+      <c r="E147" s="4">
+        <v>1</v>
+      </c>
+      <c r="F147" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -8843,9 +9287,12 @@
         </is>
       </c>
       <c r="D148" s="4">
+        <v>7</v>
+      </c>
+      <c r="E148" s="4">
         <v>2</v>
       </c>
-      <c r="E148" s="6" t="inlineStr">
+      <c r="F148" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -8899,9 +9346,12 @@
         </is>
       </c>
       <c r="D149" s="4">
+        <v>7</v>
+      </c>
+      <c r="E149" s="4">
         <v>3</v>
       </c>
-      <c r="E149" s="6" t="inlineStr">
+      <c r="F149" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -8955,9 +9405,12 @@
         </is>
       </c>
       <c r="D150" s="4">
+        <v>7</v>
+      </c>
+      <c r="E150" s="4">
         <v>4</v>
       </c>
-      <c r="E150" s="6" t="inlineStr">
+      <c r="F150" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -9011,9 +9464,12 @@
         </is>
       </c>
       <c r="D151" s="4">
+        <v>7</v>
+      </c>
+      <c r="E151" s="4">
         <v>5</v>
       </c>
-      <c r="E151" s="6" t="inlineStr">
+      <c r="F151" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -9067,9 +9523,12 @@
         </is>
       </c>
       <c r="D152" s="4">
+        <v>7</v>
+      </c>
+      <c r="E152" s="4">
         <v>6</v>
       </c>
-      <c r="E152" s="6" t="inlineStr">
+      <c r="F152" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -9125,7 +9584,10 @@
       <c r="D153" s="4">
         <v>7</v>
       </c>
-      <c r="E153" s="6" t="inlineStr">
+      <c r="E153" s="4">
+        <v>7</v>
+      </c>
+      <c r="F153" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -9181,7 +9643,10 @@
       <c r="D154" s="4">
         <v>1</v>
       </c>
-      <c r="E154" s="6" t="inlineStr">
+      <c r="E154" s="4">
+        <v>1</v>
+      </c>
+      <c r="F154" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -9237,7 +9702,10 @@
       <c r="D155" s="4">
         <v>1</v>
       </c>
-      <c r="E155" s="6" t="inlineStr">
+      <c r="E155" s="4">
+        <v>1</v>
+      </c>
+      <c r="F155" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -9300,7 +9768,10 @@
       <c r="D156" s="4">
         <v>1</v>
       </c>
-      <c r="E156" s="6" t="inlineStr">
+      <c r="E156" s="4">
+        <v>1</v>
+      </c>
+      <c r="F156" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -9363,7 +9834,10 @@
       <c r="D157" s="4">
         <v>1</v>
       </c>
-      <c r="E157" s="6" t="inlineStr">
+      <c r="E157" s="4">
+        <v>1</v>
+      </c>
+      <c r="F157" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -9432,9 +9906,12 @@
         </is>
       </c>
       <c r="D158" s="4">
-        <v>1</v>
-      </c>
-      <c r="E158" s="6" t="inlineStr">
+        <v>2</v>
+      </c>
+      <c r="E158" s="4">
+        <v>1</v>
+      </c>
+      <c r="F158" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -9497,7 +9974,10 @@
       <c r="D159" s="4">
         <v>2</v>
       </c>
-      <c r="E159" s="6" t="inlineStr">
+      <c r="E159" s="4">
+        <v>2</v>
+      </c>
+      <c r="F159" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -9558,9 +10038,12 @@
         </is>
       </c>
       <c r="D160" s="4">
-        <v>1</v>
-      </c>
-      <c r="E160" s="6" t="inlineStr">
+        <v>2</v>
+      </c>
+      <c r="E160" s="4">
+        <v>1</v>
+      </c>
+      <c r="F160" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -9631,7 +10114,10 @@
       <c r="D161" s="4">
         <v>2</v>
       </c>
-      <c r="E161" s="6" t="inlineStr">
+      <c r="E161" s="4">
+        <v>2</v>
+      </c>
+      <c r="F161" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -9702,7 +10188,10 @@
       <c r="D162" s="4">
         <v>1</v>
       </c>
-      <c r="E162" s="6" t="inlineStr">
+      <c r="E162" s="4">
+        <v>1</v>
+      </c>
+      <c r="F162" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -9795,7 +10284,10 @@
       <c r="D163" s="4">
         <v>1</v>
       </c>
-      <c r="E163" s="6" t="inlineStr">
+      <c r="E163" s="4">
+        <v>1</v>
+      </c>
+      <c r="F163" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -9866,7 +10358,10 @@
       <c r="D164" s="4">
         <v>1</v>
       </c>
-      <c r="E164" s="6" t="inlineStr">
+      <c r="E164" s="4">
+        <v>1</v>
+      </c>
+      <c r="F164" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -9936,9 +10431,12 @@
         </is>
       </c>
       <c r="D165" s="4">
-        <v>1</v>
-      </c>
-      <c r="E165" s="6" t="inlineStr">
+        <v>2</v>
+      </c>
+      <c r="E165" s="4">
+        <v>1</v>
+      </c>
+      <c r="F165" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -10010,7 +10508,10 @@
       <c r="D166" s="4">
         <v>2</v>
       </c>
-      <c r="E166" s="6" t="inlineStr">
+      <c r="E166" s="4">
+        <v>2</v>
+      </c>
+      <c r="F166" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -10080,9 +10581,12 @@
         </is>
       </c>
       <c r="D167" s="4">
-        <v>1</v>
-      </c>
-      <c r="E167" s="6" t="inlineStr">
+        <v>5</v>
+      </c>
+      <c r="E167" s="4">
+        <v>1</v>
+      </c>
+      <c r="F167" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -10136,9 +10640,12 @@
         </is>
       </c>
       <c r="D168" s="4">
+        <v>5</v>
+      </c>
+      <c r="E168" s="4">
         <v>2</v>
       </c>
-      <c r="E168" s="6" t="inlineStr">
+      <c r="F168" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -10192,9 +10699,12 @@
         </is>
       </c>
       <c r="D169" s="4">
+        <v>5</v>
+      </c>
+      <c r="E169" s="4">
         <v>3</v>
       </c>
-      <c r="E169" s="6" t="inlineStr">
+      <c r="F169" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -10248,9 +10758,12 @@
         </is>
       </c>
       <c r="D170" s="4">
+        <v>5</v>
+      </c>
+      <c r="E170" s="4">
         <v>4</v>
       </c>
-      <c r="E170" s="6" t="inlineStr">
+      <c r="F170" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -10306,7 +10819,10 @@
       <c r="D171" s="4">
         <v>5</v>
       </c>
-      <c r="E171" s="6" t="inlineStr">
+      <c r="E171" s="4">
+        <v>5</v>
+      </c>
+      <c r="F171" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -10362,7 +10878,10 @@
       <c r="D172" s="4">
         <v>1</v>
       </c>
-      <c r="E172" s="6" t="inlineStr">
+      <c r="E172" s="4">
+        <v>1</v>
+      </c>
+      <c r="F172" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -10434,7 +10953,10 @@
       <c r="D173" s="4">
         <v>1</v>
       </c>
-      <c r="E173" s="6" t="inlineStr">
+      <c r="E173" s="4">
+        <v>1</v>
+      </c>
+      <c r="F173" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -10542,7 +11064,10 @@
       <c r="D174" s="4">
         <v>1</v>
       </c>
-      <c r="E174" s="6" t="inlineStr">
+      <c r="E174" s="4">
+        <v>1</v>
+      </c>
+      <c r="F174" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -10603,9 +11128,12 @@
         </is>
       </c>
       <c r="D175" s="4">
-        <v>1</v>
-      </c>
-      <c r="E175" s="6" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="E175" s="4">
+        <v>1</v>
+      </c>
+      <c r="F175" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -10675,9 +11203,12 @@
         </is>
       </c>
       <c r="D176" s="4">
+        <v>3</v>
+      </c>
+      <c r="E176" s="4">
         <v>2</v>
       </c>
-      <c r="E176" s="6" t="inlineStr">
+      <c r="F176" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -10749,7 +11280,10 @@
       <c r="D177" s="4">
         <v>3</v>
       </c>
-      <c r="E177" s="6" t="inlineStr">
+      <c r="E177" s="4">
+        <v>3</v>
+      </c>
+      <c r="F177" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -10819,9 +11353,12 @@
         </is>
       </c>
       <c r="D178" s="4">
-        <v>1</v>
-      </c>
-      <c r="E178" s="6" t="inlineStr">
+        <v>2</v>
+      </c>
+      <c r="E178" s="4">
+        <v>1</v>
+      </c>
+      <c r="F178" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -10893,7 +11430,10 @@
       <c r="D179" s="4">
         <v>2</v>
       </c>
-      <c r="E179" s="6" t="inlineStr">
+      <c r="E179" s="4">
+        <v>2</v>
+      </c>
+      <c r="F179" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -10963,9 +11503,12 @@
         </is>
       </c>
       <c r="D180" s="4">
-        <v>1</v>
-      </c>
-      <c r="E180" s="6" t="inlineStr">
+        <v>2</v>
+      </c>
+      <c r="E180" s="4">
+        <v>1</v>
+      </c>
+      <c r="F180" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -11037,7 +11580,10 @@
       <c r="D181" s="4">
         <v>2</v>
       </c>
-      <c r="E181" s="6" t="inlineStr">
+      <c r="E181" s="4">
+        <v>2</v>
+      </c>
+      <c r="F181" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -11109,7 +11655,10 @@
       <c r="D182" s="4">
         <v>1</v>
       </c>
-      <c r="E182" s="6" t="inlineStr">
+      <c r="E182" s="4">
+        <v>1</v>
+      </c>
+      <c r="F182" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -11181,7 +11730,10 @@
       <c r="D183" s="4">
         <v>1</v>
       </c>
-      <c r="E183" s="6" t="inlineStr">
+      <c r="E183" s="4">
+        <v>1</v>
+      </c>
+      <c r="F183" s="6" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -11235,112 +11787,147 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="105">
+  <mergeCells count="140">
     <mergeCell ref="A2:A6"/>
     <mergeCell ref="B2:B6"/>
     <mergeCell ref="C2:C6"/>
+    <mergeCell ref="D2:D6"/>
     <mergeCell ref="A7:A10"/>
     <mergeCell ref="B7:B10"/>
     <mergeCell ref="C7:C10"/>
+    <mergeCell ref="D7:D10"/>
     <mergeCell ref="A12:A15"/>
     <mergeCell ref="B12:B15"/>
     <mergeCell ref="C12:C15"/>
+    <mergeCell ref="D12:D15"/>
     <mergeCell ref="A16:A18"/>
     <mergeCell ref="B16:B18"/>
     <mergeCell ref="C16:C18"/>
+    <mergeCell ref="D16:D18"/>
     <mergeCell ref="A19:A21"/>
     <mergeCell ref="B19:B21"/>
     <mergeCell ref="C19:C21"/>
+    <mergeCell ref="D19:D21"/>
     <mergeCell ref="A23:A27"/>
     <mergeCell ref="B23:B27"/>
     <mergeCell ref="C23:C27"/>
+    <mergeCell ref="D23:D27"/>
     <mergeCell ref="A29:A33"/>
     <mergeCell ref="B29:B33"/>
     <mergeCell ref="C29:C33"/>
+    <mergeCell ref="D29:D33"/>
     <mergeCell ref="A34:A35"/>
     <mergeCell ref="B34:B35"/>
     <mergeCell ref="C34:C35"/>
+    <mergeCell ref="D34:D35"/>
     <mergeCell ref="A40:A41"/>
     <mergeCell ref="B40:B41"/>
     <mergeCell ref="C40:C41"/>
+    <mergeCell ref="D40:D41"/>
     <mergeCell ref="A44:A46"/>
     <mergeCell ref="B44:B46"/>
     <mergeCell ref="C44:C46"/>
+    <mergeCell ref="D44:D46"/>
     <mergeCell ref="A51:A52"/>
     <mergeCell ref="B51:B52"/>
     <mergeCell ref="C51:C52"/>
+    <mergeCell ref="D51:D52"/>
     <mergeCell ref="A57:A59"/>
     <mergeCell ref="B57:B59"/>
     <mergeCell ref="C57:C59"/>
+    <mergeCell ref="D57:D59"/>
     <mergeCell ref="A65:A69"/>
     <mergeCell ref="B65:B69"/>
     <mergeCell ref="C65:C69"/>
+    <mergeCell ref="D65:D69"/>
     <mergeCell ref="A71:A74"/>
     <mergeCell ref="B71:B74"/>
     <mergeCell ref="C71:C74"/>
+    <mergeCell ref="D71:D74"/>
     <mergeCell ref="A77:A78"/>
     <mergeCell ref="B77:B78"/>
     <mergeCell ref="C77:C78"/>
+    <mergeCell ref="D77:D78"/>
     <mergeCell ref="A80:A82"/>
     <mergeCell ref="B80:B82"/>
     <mergeCell ref="C80:C82"/>
+    <mergeCell ref="D80:D82"/>
     <mergeCell ref="A83:A87"/>
     <mergeCell ref="B83:B87"/>
     <mergeCell ref="C83:C87"/>
+    <mergeCell ref="D83:D87"/>
     <mergeCell ref="A89:A92"/>
     <mergeCell ref="B89:B92"/>
     <mergeCell ref="C89:C92"/>
+    <mergeCell ref="D89:D92"/>
     <mergeCell ref="A93:A94"/>
     <mergeCell ref="B93:B94"/>
     <mergeCell ref="C93:C94"/>
+    <mergeCell ref="D93:D94"/>
     <mergeCell ref="A103:A105"/>
     <mergeCell ref="B103:B105"/>
     <mergeCell ref="C103:C105"/>
+    <mergeCell ref="D103:D105"/>
     <mergeCell ref="A110:A111"/>
     <mergeCell ref="B110:B111"/>
     <mergeCell ref="C110:C111"/>
+    <mergeCell ref="D110:D111"/>
     <mergeCell ref="A112:A113"/>
     <mergeCell ref="B112:B113"/>
     <mergeCell ref="C112:C113"/>
+    <mergeCell ref="D112:D113"/>
     <mergeCell ref="A123:A125"/>
     <mergeCell ref="B123:B125"/>
     <mergeCell ref="C123:C125"/>
+    <mergeCell ref="D123:D125"/>
     <mergeCell ref="A126:A130"/>
     <mergeCell ref="B126:B130"/>
     <mergeCell ref="C126:C130"/>
+    <mergeCell ref="D126:D130"/>
     <mergeCell ref="A131:A132"/>
     <mergeCell ref="B131:B132"/>
     <mergeCell ref="C131:C132"/>
+    <mergeCell ref="D131:D132"/>
     <mergeCell ref="A134:A135"/>
     <mergeCell ref="B134:B135"/>
     <mergeCell ref="C134:C135"/>
+    <mergeCell ref="D134:D135"/>
     <mergeCell ref="A141:A142"/>
     <mergeCell ref="B141:B142"/>
     <mergeCell ref="C141:C142"/>
+    <mergeCell ref="D141:D142"/>
     <mergeCell ref="A147:A153"/>
     <mergeCell ref="B147:B153"/>
     <mergeCell ref="C147:C153"/>
+    <mergeCell ref="D147:D153"/>
     <mergeCell ref="A158:A159"/>
     <mergeCell ref="B158:B159"/>
     <mergeCell ref="C158:C159"/>
+    <mergeCell ref="D158:D159"/>
     <mergeCell ref="A160:A161"/>
     <mergeCell ref="B160:B161"/>
     <mergeCell ref="C160:C161"/>
+    <mergeCell ref="D160:D161"/>
     <mergeCell ref="A165:A166"/>
     <mergeCell ref="B165:B166"/>
     <mergeCell ref="C165:C166"/>
+    <mergeCell ref="D165:D166"/>
     <mergeCell ref="A167:A171"/>
     <mergeCell ref="B167:B171"/>
     <mergeCell ref="C167:C171"/>
+    <mergeCell ref="D167:D171"/>
     <mergeCell ref="A175:A177"/>
     <mergeCell ref="B175:B177"/>
     <mergeCell ref="C175:C177"/>
+    <mergeCell ref="D175:D177"/>
     <mergeCell ref="A178:A179"/>
     <mergeCell ref="B178:B179"/>
     <mergeCell ref="C178:C179"/>
+    <mergeCell ref="D178:D179"/>
     <mergeCell ref="A180:A181"/>
     <mergeCell ref="B180:B181"/>
     <mergeCell ref="C180:C181"/>
+    <mergeCell ref="D180:D181"/>
   </mergeCells>
   <printOptions gridLines="1" gridLinesSet="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>